<commit_message>
Changes required done till milestone 3
</commit_message>
<xml_diff>
--- a/templates/Unit_Test_Plan_Filled.xlsx
+++ b/templates/Unit_Test_Plan_Filled.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30131"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30228"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/bc20060aec94d36e/Desktop/Multi-AI-Agent-Coding-Assistant/templates/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/bc20060aec94d36e/Desktop/Multi-AI-Agent-Coding-Assistant - Copy(freebuff)/templates/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="15" documentId="11_EC6CC44CF3BCB99BC811487D28D304D83B3C6462" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{63F26C66-0DB2-423B-8A77-7A80A5C99340}"/>
+  <xr:revisionPtr revIDLastSave="9" documentId="11_4F6DF0643C42D0055C65FF212A699F98B7A5A8A3" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{4C69E7E3-7A4E-4993-BDF3-4657D03BC30E}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="126" uniqueCount="125">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="198" uniqueCount="193">
   <si>
     <t>Sl: No:</t>
   </si>
@@ -395,6 +395,210 @@
   </si>
   <si>
     <t>Validation message displayed successfully.</t>
+  </si>
+  <si>
+    <t>TC-021</t>
+  </si>
+  <si>
+    <t>Quick Actions</t>
+  </si>
+  <si>
+    <t>Ask-first flow</t>
+  </si>
+  <si>
+    <t>Click each quick action.</t>
+  </si>
+  <si>
+    <t>A question prompt appears and nothing runs until the user types.</t>
+  </si>
+  <si>
+    <t>Quick actions ask first, no auto-submit.</t>
+  </si>
+  <si>
+    <t>TC-022</t>
+  </si>
+  <si>
+    <t>Upload Dedupe</t>
+  </si>
+  <si>
+    <t>Duplicate upload</t>
+  </si>
+  <si>
+    <t>Upload the same file twice.</t>
+  </si>
+  <si>
+    <t>Only one entry in My Files.</t>
+  </si>
+  <si>
+    <t>File appears exactly once.</t>
+  </si>
+  <si>
+    <t>TC-023</t>
+  </si>
+  <si>
+    <t>File Routing</t>
+  </si>
+  <si>
+    <t>Analyse it</t>
+  </si>
+  <si>
+    <t>Attach a file and send 'analyse it'.</t>
+  </si>
+  <si>
+    <t>Routed to Code Analysis Agent.</t>
+  </si>
+  <si>
+    <t>Analysis performed on the attached file.</t>
+  </si>
+  <si>
+    <t>TC-024</t>
+  </si>
+  <si>
+    <t>Review it</t>
+  </si>
+  <si>
+    <t>Attach a file and send 'review it'.</t>
+  </si>
+  <si>
+    <t>Review performed on the attached file.</t>
+  </si>
+  <si>
+    <t>TC-025</t>
+  </si>
+  <si>
+    <t>Attach a file and send 'generate documentation'.</t>
+  </si>
+  <si>
+    <t>Routed to Documentation Agent.</t>
+  </si>
+  <si>
+    <t>Documentation generated from the attached file.</t>
+  </si>
+  <si>
+    <t>TC-026</t>
+  </si>
+  <si>
+    <t>Analytics KPIs</t>
+  </si>
+  <si>
+    <t>Exact numbers</t>
+  </si>
+  <si>
+    <t>Open Analytics with no executions.</t>
+  </si>
+  <si>
+    <t>Success rate shows 0%, conversations count real chats only.</t>
+  </si>
+  <si>
+    <t>Dashboard numbers are exact.</t>
+  </si>
+  <si>
+    <t>TC-027</t>
+  </si>
+  <si>
+    <t>Files Page</t>
+  </si>
+  <si>
+    <t>Single save</t>
+  </si>
+  <si>
+    <t>Upload a file on My Files and rerun the page.</t>
+  </si>
+  <si>
+    <t>The file is saved exactly once.</t>
+  </si>
+  <si>
+    <t>No duplicate entries created.</t>
+  </si>
+  <si>
+    <t>TC-028</t>
+  </si>
+  <si>
+    <t>Chat History</t>
+  </si>
+  <si>
+    <t>Search</t>
+  </si>
+  <si>
+    <t>Search past conversations and messages.</t>
+  </si>
+  <si>
+    <t>Matching chats and message hits listed.</t>
+  </si>
+  <si>
+    <t>Search works correctly.</t>
+  </si>
+  <si>
+    <t>TC-029</t>
+  </si>
+  <si>
+    <t>Conversation Export</t>
+  </si>
+  <si>
+    <t>Export</t>
+  </si>
+  <si>
+    <t>Export a single conversation from Chat History.</t>
+  </si>
+  <si>
+    <t>Conversation downloads as a file.</t>
+  </si>
+  <si>
+    <t>Export verified successfully.</t>
+  </si>
+  <si>
+    <t>TC-030</t>
+  </si>
+  <si>
+    <t>Legal Pages</t>
+  </si>
+  <si>
+    <t>Render</t>
+  </si>
+  <si>
+    <t>Open Terms, Privacy, Help and What's new.</t>
+  </si>
+  <si>
+    <t>Each page renders without errors.</t>
+  </si>
+  <si>
+    <t>Legal pages render correctly.</t>
+  </si>
+  <si>
+    <t>TC-031</t>
+  </si>
+  <si>
+    <t>Settings</t>
+  </si>
+  <si>
+    <t>Dark-only + English</t>
+  </si>
+  <si>
+    <t>Open Settings and try to change theme/language.</t>
+  </si>
+  <si>
+    <t>Only text size and other preferences available.</t>
+  </si>
+  <si>
+    <t>App stays dark and in English.</t>
+  </si>
+  <si>
+    <t>TC-032</t>
+  </si>
+  <si>
+    <t>Uploader Reset</t>
+  </si>
+  <si>
+    <t>No errors</t>
+  </si>
+  <si>
+    <t>Upload a file, send a message, then upload again.</t>
+  </si>
+  <si>
+    <t>No Streamlit exceptions; files not re-saved.</t>
+  </si>
+  <si>
+    <t>Uploader resets cleanly.</t>
   </si>
 </sst>
 </file>
@@ -789,15 +993,15 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:F21"/>
+  <dimension ref="A1:F33"/>
   <sheetFormatPr defaultRowHeight="13.2" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="9.109375" customWidth="1"/>
     <col min="2" max="2" width="19.88671875" customWidth="1"/>
     <col min="3" max="3" width="20.21875" customWidth="1"/>
-    <col min="4" max="4" width="25.88671875" customWidth="1"/>
-    <col min="5" max="5" width="24.109375" customWidth="1"/>
-    <col min="6" max="6" width="36.33203125" customWidth="1"/>
+    <col min="4" max="4" width="41.5546875" customWidth="1"/>
+    <col min="5" max="5" width="53.77734375" customWidth="1"/>
+    <col min="6" max="6" width="42.21875" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:6" ht="31.5" customHeight="1" x14ac:dyDescent="0.25">
@@ -920,7 +1124,7 @@
         <v>35</v>
       </c>
     </row>
-    <row r="7" spans="1:6" ht="14.4" x14ac:dyDescent="0.3">
+    <row r="7" spans="1:6" ht="14.4" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A7" s="3" t="s">
         <v>36</v>
       </c>
@@ -940,7 +1144,7 @@
         <v>41</v>
       </c>
     </row>
-    <row r="8" spans="1:6" ht="14.4" x14ac:dyDescent="0.3">
+    <row r="8" spans="1:6" ht="14.4" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A8" s="3" t="s">
         <v>42</v>
       </c>
@@ -960,7 +1164,7 @@
         <v>47</v>
       </c>
     </row>
-    <row r="9" spans="1:6" ht="14.4" x14ac:dyDescent="0.3">
+    <row r="9" spans="1:6" ht="14.4" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A9" s="3" t="s">
         <v>48</v>
       </c>
@@ -980,7 +1184,7 @@
         <v>53</v>
       </c>
     </row>
-    <row r="10" spans="1:6" ht="14.4" x14ac:dyDescent="0.3">
+    <row r="10" spans="1:6" ht="14.4" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A10" s="3" t="s">
         <v>54</v>
       </c>
@@ -1000,7 +1204,7 @@
         <v>59</v>
       </c>
     </row>
-    <row r="11" spans="1:6" ht="14.4" x14ac:dyDescent="0.3">
+    <row r="11" spans="1:6" ht="14.4" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A11" s="3" t="s">
         <v>60</v>
       </c>
@@ -1020,7 +1224,7 @@
         <v>65</v>
       </c>
     </row>
-    <row r="12" spans="1:6" ht="14.4" x14ac:dyDescent="0.3">
+    <row r="12" spans="1:6" ht="14.4" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A12" s="3" t="s">
         <v>66</v>
       </c>
@@ -1040,7 +1244,7 @@
         <v>71</v>
       </c>
     </row>
-    <row r="13" spans="1:6" ht="14.4" x14ac:dyDescent="0.3">
+    <row r="13" spans="1:6" ht="14.4" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A13" s="3" t="s">
         <v>72</v>
       </c>
@@ -1060,7 +1264,7 @@
         <v>77</v>
       </c>
     </row>
-    <row r="14" spans="1:6" ht="14.4" x14ac:dyDescent="0.3">
+    <row r="14" spans="1:6" ht="14.4" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A14" s="3" t="s">
         <v>78</v>
       </c>
@@ -1080,7 +1284,7 @@
         <v>83</v>
       </c>
     </row>
-    <row r="15" spans="1:6" ht="14.4" x14ac:dyDescent="0.3">
+    <row r="15" spans="1:6" ht="14.4" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A15" s="3" t="s">
         <v>84</v>
       </c>
@@ -1100,7 +1304,7 @@
         <v>89</v>
       </c>
     </row>
-    <row r="16" spans="1:6" ht="14.4" x14ac:dyDescent="0.3">
+    <row r="16" spans="1:6" ht="14.4" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A16" s="3" t="s">
         <v>90</v>
       </c>
@@ -1120,7 +1324,7 @@
         <v>95</v>
       </c>
     </row>
-    <row r="17" spans="1:6" ht="14.4" x14ac:dyDescent="0.3">
+    <row r="17" spans="1:6" ht="14.4" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A17" s="3" t="s">
         <v>96</v>
       </c>
@@ -1140,7 +1344,7 @@
         <v>101</v>
       </c>
     </row>
-    <row r="18" spans="1:6" ht="14.4" x14ac:dyDescent="0.3">
+    <row r="18" spans="1:6" ht="14.4" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A18" s="3" t="s">
         <v>102</v>
       </c>
@@ -1160,7 +1364,7 @@
         <v>107</v>
       </c>
     </row>
-    <row r="19" spans="1:6" ht="14.4" x14ac:dyDescent="0.3">
+    <row r="19" spans="1:6" ht="14.4" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A19" s="3" t="s">
         <v>108</v>
       </c>
@@ -1180,7 +1384,7 @@
         <v>113</v>
       </c>
     </row>
-    <row r="20" spans="1:6" ht="14.4" x14ac:dyDescent="0.3">
+    <row r="20" spans="1:6" ht="14.4" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A20" s="3" t="s">
         <v>114</v>
       </c>
@@ -1200,7 +1404,7 @@
         <v>118</v>
       </c>
     </row>
-    <row r="21" spans="1:6" ht="14.4" x14ac:dyDescent="0.3">
+    <row r="21" spans="1:6" ht="14.4" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A21" s="3" t="s">
         <v>119</v>
       </c>
@@ -1218,6 +1422,246 @@
       </c>
       <c r="F21" s="3" t="s">
         <v>124</v>
+      </c>
+    </row>
+    <row r="22" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A22" t="s">
+        <v>125</v>
+      </c>
+      <c r="B22" t="s">
+        <v>126</v>
+      </c>
+      <c r="C22" t="s">
+        <v>127</v>
+      </c>
+      <c r="D22" t="s">
+        <v>128</v>
+      </c>
+      <c r="E22" t="s">
+        <v>129</v>
+      </c>
+      <c r="F22" t="s">
+        <v>130</v>
+      </c>
+    </row>
+    <row r="23" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A23" t="s">
+        <v>131</v>
+      </c>
+      <c r="B23" t="s">
+        <v>132</v>
+      </c>
+      <c r="C23" t="s">
+        <v>133</v>
+      </c>
+      <c r="D23" t="s">
+        <v>134</v>
+      </c>
+      <c r="E23" t="s">
+        <v>135</v>
+      </c>
+      <c r="F23" t="s">
+        <v>136</v>
+      </c>
+    </row>
+    <row r="24" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A24" t="s">
+        <v>137</v>
+      </c>
+      <c r="B24" t="s">
+        <v>138</v>
+      </c>
+      <c r="C24" t="s">
+        <v>139</v>
+      </c>
+      <c r="D24" t="s">
+        <v>140</v>
+      </c>
+      <c r="E24" t="s">
+        <v>141</v>
+      </c>
+      <c r="F24" t="s">
+        <v>142</v>
+      </c>
+    </row>
+    <row r="25" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A25" t="s">
+        <v>143</v>
+      </c>
+      <c r="B25" t="s">
+        <v>138</v>
+      </c>
+      <c r="C25" t="s">
+        <v>144</v>
+      </c>
+      <c r="D25" t="s">
+        <v>145</v>
+      </c>
+      <c r="E25" t="s">
+        <v>141</v>
+      </c>
+      <c r="F25" t="s">
+        <v>146</v>
+      </c>
+    </row>
+    <row r="26" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A26" t="s">
+        <v>147</v>
+      </c>
+      <c r="B26" t="s">
+        <v>138</v>
+      </c>
+      <c r="C26" t="s">
+        <v>44</v>
+      </c>
+      <c r="D26" t="s">
+        <v>148</v>
+      </c>
+      <c r="E26" t="s">
+        <v>149</v>
+      </c>
+      <c r="F26" t="s">
+        <v>150</v>
+      </c>
+    </row>
+    <row r="27" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A27" t="s">
+        <v>151</v>
+      </c>
+      <c r="B27" t="s">
+        <v>152</v>
+      </c>
+      <c r="C27" t="s">
+        <v>153</v>
+      </c>
+      <c r="D27" t="s">
+        <v>154</v>
+      </c>
+      <c r="E27" t="s">
+        <v>155</v>
+      </c>
+      <c r="F27" t="s">
+        <v>156</v>
+      </c>
+    </row>
+    <row r="28" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A28" t="s">
+        <v>157</v>
+      </c>
+      <c r="B28" t="s">
+        <v>158</v>
+      </c>
+      <c r="C28" t="s">
+        <v>159</v>
+      </c>
+      <c r="D28" t="s">
+        <v>160</v>
+      </c>
+      <c r="E28" t="s">
+        <v>161</v>
+      </c>
+      <c r="F28" t="s">
+        <v>162</v>
+      </c>
+    </row>
+    <row r="29" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A29" t="s">
+        <v>163</v>
+      </c>
+      <c r="B29" t="s">
+        <v>164</v>
+      </c>
+      <c r="C29" t="s">
+        <v>165</v>
+      </c>
+      <c r="D29" t="s">
+        <v>166</v>
+      </c>
+      <c r="E29" t="s">
+        <v>167</v>
+      </c>
+      <c r="F29" t="s">
+        <v>168</v>
+      </c>
+    </row>
+    <row r="30" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A30" t="s">
+        <v>169</v>
+      </c>
+      <c r="B30" t="s">
+        <v>170</v>
+      </c>
+      <c r="C30" t="s">
+        <v>171</v>
+      </c>
+      <c r="D30" t="s">
+        <v>172</v>
+      </c>
+      <c r="E30" t="s">
+        <v>173</v>
+      </c>
+      <c r="F30" t="s">
+        <v>174</v>
+      </c>
+    </row>
+    <row r="31" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A31" t="s">
+        <v>175</v>
+      </c>
+      <c r="B31" t="s">
+        <v>176</v>
+      </c>
+      <c r="C31" t="s">
+        <v>177</v>
+      </c>
+      <c r="D31" t="s">
+        <v>178</v>
+      </c>
+      <c r="E31" t="s">
+        <v>179</v>
+      </c>
+      <c r="F31" t="s">
+        <v>180</v>
+      </c>
+    </row>
+    <row r="32" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A32" t="s">
+        <v>181</v>
+      </c>
+      <c r="B32" t="s">
+        <v>182</v>
+      </c>
+      <c r="C32" t="s">
+        <v>183</v>
+      </c>
+      <c r="D32" t="s">
+        <v>184</v>
+      </c>
+      <c r="E32" t="s">
+        <v>185</v>
+      </c>
+      <c r="F32" t="s">
+        <v>186</v>
+      </c>
+    </row>
+    <row r="33" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A33" t="s">
+        <v>187</v>
+      </c>
+      <c r="B33" t="s">
+        <v>188</v>
+      </c>
+      <c r="C33" t="s">
+        <v>189</v>
+      </c>
+      <c r="D33" t="s">
+        <v>190</v>
+      </c>
+      <c r="E33" t="s">
+        <v>191</v>
+      </c>
+      <c r="F33" t="s">
+        <v>192</v>
       </c>
     </row>
   </sheetData>

</xml_diff>